<commit_message>
Update set-04 and set-05 task boards to match template
</commit_message>
<xml_diff>
--- a/set-04/Ecommerce-Intern-Debug-Task-Board-Set-04.xlsx
+++ b/set-04/Ecommerce-Intern-Debug-Task-Board-Set-04.xlsx
@@ -5,102 +5,111 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Task Board" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="How To Do Task" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Status Meaning" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Test Guide" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="41">
-  <si>
-    <t>Project</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="69">
+  <si>
+    <t>Intern</t>
   </si>
   <si>
     <t>Task ID</t>
   </si>
   <si>
-    <t>Task Title</t>
-  </si>
-  <si>
-    <t>Folder</t>
-  </si>
-  <si>
-    <t>Files</t>
-  </si>
-  <si>
-    <t>Debug Focus</t>
+    <t>File</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>Step / focus</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
+    <t>Tests</t>
+  </si>
+  <si>
+    <t>PR Link</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>VelvetCart</t>
   </si>
   <si>
     <t>07-01</t>
   </si>
   <si>
-    <t>Selection Toggle</t>
-  </si>
-  <si>
     <t>project-07-velvetcart/task-01-selection-toggle</t>
   </si>
   <si>
-    <t>index.html, styles.css, script.js</t>
-  </si>
-  <si>
-    <t>Selected option should update label and active state, but the selector and dataset key are wrong.</t>
+    <t>Selection toggle</t>
+  </si>
+  <si>
+    <t>Fix selector, active class handling, and dataset lookup.</t>
   </si>
   <si>
     <t>Not Started</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>07-02</t>
   </si>
   <si>
-    <t>Count Updater</t>
-  </si>
-  <si>
     <t>project-07-velvetcart/task-02-count-updater</t>
   </si>
   <si>
-    <t>Button clicks should increase the visible count numerically, but the wrong element ID and string math are used.</t>
+    <t>Cart count update</t>
+  </si>
+  <si>
+    <t>Fix wrong target element and numeric increment logic.</t>
   </si>
   <si>
     <t>07-03</t>
   </si>
   <si>
-    <t>Live Filter</t>
-  </si>
-  <si>
     <t>project-07-velvetcart/task-03-live-filter</t>
   </si>
   <si>
-    <t>List should filter while typing, but the code uses the wrong event and hides matches instead of non-matches.</t>
+    <t>Live filter</t>
+  </si>
+  <si>
+    <t>Show matching products and hide non-matches using the correct comparison.</t>
   </si>
   <si>
     <t>07-04</t>
   </si>
   <si>
-    <t>Gallery Preview</t>
-  </si>
-  <si>
     <t>project-07-velvetcart/task-04-gallery-preview</t>
   </si>
   <si>
-    <t>Thumbnail clicks should update the main image, but the selector and dataset property do not match the HTML.</t>
+    <t>Gallery preview</t>
+  </si>
+  <si>
+    <t>Fix thumbnail selector and image dataset property.</t>
   </si>
   <si>
     <t>07-05</t>
   </si>
   <si>
-    <t>Progress Bar</t>
-  </si>
-  <si>
     <t>project-07-velvetcart/task-05-progress-bar</t>
   </si>
   <si>
-    <t>Progress should fill based on the percentage, but the width is missing a CSS unit.</t>
+    <t>Promo progress</t>
+  </si>
+  <si>
+    <t>Convert progress into a valid CSS width percentage.</t>
   </si>
   <si>
     <t>NestNook</t>
@@ -134,6 +143,84 @@
   </si>
   <si>
     <t>project-08-nestnook/task-05-progress-bar</t>
+  </si>
+  <si>
+    <t>Section</t>
+  </si>
+  <si>
+    <t>Instructions</t>
+  </si>
+  <si>
+    <t>Overview</t>
+  </si>
+  <si>
+    <t>This workbook tracks 10 front-end e-commerce debugging tasks across 2 projects. Each row points to one task folder containing HTML, CSS, and JavaScript with intentional bugs.</t>
+  </si>
+  <si>
+    <t>How to work</t>
+  </si>
+  <si>
+    <t>Open one task in the browser, reproduce the issue, inspect the code, fix the root cause, and record your progress in the Task Board.</t>
+  </si>
+  <si>
+    <t>Expected output</t>
+  </si>
+  <si>
+    <t>The goal is to debug the current implementation, not rebuild the page from scratch. Update Status, add notes, and paste a PR link when work is submitted.</t>
+  </si>
+  <si>
+    <t>Meaning (for the Task Board)</t>
+  </si>
+  <si>
+    <t>No changes made yet.</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Task is being debugged locally.</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Fix is complete locally and ready for review.</t>
+  </si>
+  <si>
+    <t>PR Submitted</t>
+  </si>
+  <si>
+    <t>Pull request has been opened and is waiting for review or merge.</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>What it means</t>
+  </si>
+  <si>
+    <t>Broken behavior reproduced</t>
+  </si>
+  <si>
+    <t>You confirmed the bug in the browser and understand what needs to be fixed.</t>
+  </si>
+  <si>
+    <t>Fix verified</t>
+  </si>
+  <si>
+    <t>The page behaves correctly after your code changes.</t>
+  </si>
+  <si>
+    <t>Notes updated</t>
+  </si>
+  <si>
+    <t>Use the Notes column to document what was wrong and how you fixed it.</t>
+  </si>
+  <si>
+    <t>PR Link added</t>
+  </si>
+  <si>
+    <t>Paste the GitHub pull request URL after opening your PR.</t>
   </si>
 </sst>
 </file>
@@ -520,19 +607,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="70" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="42" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="44" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -545,253 +634,476 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="E7" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="F7" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
         <v>22</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
         <v>30</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>29</v>
+      <c r="F11" t="s">
+        <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="G2:G11">
-      <formula1>"Not Started,In Progress,Done,Reviewed"</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="F2:F11">
+      <formula1>"Not Started,In Progress,Done,PR Submitted"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="22" style="1" customWidth="1"/>
+    <col min="2" max="2" width="88" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="70" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="76" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Match set-04 and set-05 workbooks to board format
</commit_message>
<xml_diff>
--- a/set-04/Ecommerce-Intern-Debug-Task-Board-Set-04.xlsx
+++ b/set-04/Ecommerce-Intern-Debug-Task-Board-Set-04.xlsx
@@ -5,41 +5,37 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Task Board" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="How To Do Task" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Status Meaning" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Test Guide" state="visible" r:id="rId7"/>
+    <sheet sheetId="2" name="Guide" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Projects" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="69">
-  <si>
-    <t>Intern</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="57">
+  <si>
+    <t>Project</t>
   </si>
   <si>
     <t>Task ID</t>
   </si>
   <si>
-    <t>File</t>
-  </si>
-  <si>
-    <t>Function</t>
-  </si>
-  <si>
-    <t>Step / focus</t>
+    <t>Task Title</t>
+  </si>
+  <si>
+    <t>Folder</t>
+  </si>
+  <si>
+    <t>Files</t>
+  </si>
+  <si>
+    <t>Debug Focus</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>Tests</t>
-  </si>
-  <si>
-    <t>PR Link</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -49,13 +45,16 @@
     <t>07-01</t>
   </si>
   <si>
+    <t>Selection Toggle</t>
+  </si>
+  <si>
     <t>project-07-velvetcart/task-01-selection-toggle</t>
   </si>
   <si>
-    <t>Selection toggle</t>
-  </si>
-  <si>
-    <t>Fix selector, active class handling, and dataset lookup.</t>
+    <t>index.html, styles.css, script.js</t>
+  </si>
+  <si>
+    <t>Selected option should update label and active state, but the selector and dataset key are wrong.</t>
   </si>
   <si>
     <t>Not Started</t>
@@ -67,49 +66,49 @@
     <t>07-02</t>
   </si>
   <si>
+    <t>Count Updater</t>
+  </si>
+  <si>
     <t>project-07-velvetcart/task-02-count-updater</t>
   </si>
   <si>
-    <t>Cart count update</t>
-  </si>
-  <si>
-    <t>Fix wrong target element and numeric increment logic.</t>
+    <t>Button clicks should increase the visible count numerically, but the wrong element ID and string math are used.</t>
   </si>
   <si>
     <t>07-03</t>
   </si>
   <si>
+    <t>Live Filter</t>
+  </si>
+  <si>
     <t>project-07-velvetcart/task-03-live-filter</t>
   </si>
   <si>
-    <t>Live filter</t>
-  </si>
-  <si>
-    <t>Show matching products and hide non-matches using the correct comparison.</t>
+    <t>List should filter while typing, but the code uses the wrong event and hides matches instead of non-matches.</t>
   </si>
   <si>
     <t>07-04</t>
   </si>
   <si>
+    <t>Gallery Preview</t>
+  </si>
+  <si>
     <t>project-07-velvetcart/task-04-gallery-preview</t>
   </si>
   <si>
-    <t>Gallery preview</t>
-  </si>
-  <si>
-    <t>Fix thumbnail selector and image dataset property.</t>
+    <t>Thumbnail clicks should update the main image, but the selector and dataset property do not match the HTML.</t>
   </si>
   <si>
     <t>07-05</t>
   </si>
   <si>
+    <t>Progress Bar</t>
+  </si>
+  <si>
     <t>project-07-velvetcart/task-05-progress-bar</t>
   </si>
   <si>
-    <t>Promo progress</t>
-  </si>
-  <si>
-    <t>Convert progress into a valid CSS width percentage.</t>
+    <t>Progress should fill based on the percentage, but the width is missing a CSS unit.</t>
   </si>
   <si>
     <t>NestNook</t>
@@ -148,79 +147,43 @@
     <t>Section</t>
   </si>
   <si>
-    <t>Instructions</t>
-  </si>
-  <si>
-    <t>Overview</t>
-  </si>
-  <si>
-    <t>This workbook tracks 10 front-end e-commerce debugging tasks across 2 projects. Each row points to one task folder containing HTML, CSS, and JavaScript with intentional bugs.</t>
-  </si>
-  <si>
-    <t>How to work</t>
-  </si>
-  <si>
-    <t>Open one task in the browser, reproduce the issue, inspect the code, fix the root cause, and record your progress in the Task Board.</t>
-  </si>
-  <si>
-    <t>Expected output</t>
-  </si>
-  <si>
-    <t>The goal is to debug the current implementation, not rebuild the page from scratch. Update Status, add notes, and paste a PR link when work is submitted.</t>
-  </si>
-  <si>
-    <t>Meaning (for the Task Board)</t>
-  </si>
-  <si>
-    <t>No changes made yet.</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Task is being debugged locally.</t>
-  </si>
-  <si>
-    <t>Done</t>
-  </si>
-  <si>
-    <t>Fix is complete locally and ready for review.</t>
-  </si>
-  <si>
-    <t>PR Submitted</t>
-  </si>
-  <si>
-    <t>Pull request has been opened and is waiting for review or merge.</t>
-  </si>
-  <si>
-    <t>Result</t>
-  </si>
-  <si>
-    <t>What it means</t>
-  </si>
-  <si>
-    <t>Broken behavior reproduced</t>
-  </si>
-  <si>
-    <t>You confirmed the bug in the browser and understand what needs to be fixed.</t>
-  </si>
-  <si>
-    <t>Fix verified</t>
-  </si>
-  <si>
-    <t>The page behaves correctly after your code changes.</t>
-  </si>
-  <si>
-    <t>Notes updated</t>
-  </si>
-  <si>
-    <t>Use the Notes column to document what was wrong and how you fixed it.</t>
-  </si>
-  <si>
-    <t>PR Link added</t>
-  </si>
-  <si>
-    <t>Paste the GitHub pull request URL after opening your PR.</t>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>What this pack is</t>
+  </si>
+  <si>
+    <t>This workbook tracks 2 e-commerce projects with 10 debugging tasks total. Each task points to a small front-end folder with intentional bugs.</t>
+  </si>
+  <si>
+    <t>How to use it</t>
+  </si>
+  <si>
+    <t>Open one task folder at a time, run the page in a browser, reproduce the issue, inspect the code, and fix the root cause.</t>
+  </si>
+  <si>
+    <t>Expected skills</t>
+  </si>
+  <si>
+    <t>DOM selection, event handling, state updates, conditional logic, filtering, class toggling, and small HTML/CSS/JavaScript debugging.</t>
+  </si>
+  <si>
+    <t>Suggested rule</t>
+  </si>
+  <si>
+    <t>Keep the feature intent the same. The goal is to debug the existing code, not replace the whole task with a brand-new build.</t>
+  </si>
+  <si>
+    <t>Theme</t>
+  </si>
+  <si>
+    <t>Task Count</t>
+  </si>
+  <si>
+    <t>Fashion accessories storefront</t>
+  </si>
+  <si>
+    <t>Home decor storefront</t>
   </si>
 </sst>
 </file>
@@ -607,21 +570,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="44" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="42" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
-    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="52" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="70" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -631,13 +593,13 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -646,42 +608,36 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
@@ -689,28 +645,25 @@
       <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
       </c>
       <c r="H3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -718,28 +671,25 @@
       <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>15</v>
       </c>
       <c r="H4" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>24</v>
@@ -747,28 +697,25 @@
       <c r="C5" t="s">
         <v>25</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>14</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
       </c>
       <c r="H5" t="s">
         <v>15</v>
       </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
         <v>28</v>
@@ -776,26 +723,23 @@
       <c r="C6" t="s">
         <v>29</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>14</v>
-      </c>
-      <c r="G6" t="s">
-        <v>15</v>
       </c>
       <c r="H6" t="s">
         <v>15</v>
       </c>
-      <c r="I6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -803,28 +747,25 @@
         <v>33</v>
       </c>
       <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>14</v>
-      </c>
-      <c r="G7" t="s">
-        <v>15</v>
       </c>
       <c r="H7" t="s">
         <v>15</v>
       </c>
-      <c r="I7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -832,28 +773,25 @@
         <v>35</v>
       </c>
       <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>14</v>
-      </c>
-      <c r="G8" t="s">
-        <v>15</v>
       </c>
       <c r="H8" t="s">
         <v>15</v>
       </c>
-      <c r="I8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -861,28 +799,25 @@
         <v>37</v>
       </c>
       <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>15</v>
       </c>
       <c r="H9" t="s">
         <v>15</v>
       </c>
-      <c r="I9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -890,28 +825,25 @@
         <v>39</v>
       </c>
       <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>14</v>
-      </c>
-      <c r="G10" t="s">
-        <v>15</v>
       </c>
       <c r="H10" t="s">
         <v>15</v>
       </c>
-      <c r="I10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -919,31 +851,28 @@
         <v>41</v>
       </c>
       <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>14</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
       </c>
       <c r="H11" t="s">
         <v>15</v>
       </c>
-      <c r="I11" t="s">
-        <v>15</v>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F11">
-      <formula1>"Not Started,In Progress,Done,PR Submitted"</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="G2:G11">
+      <formula1>"Not Started,In Progress,Done,Reviewed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -953,15 +882,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" style="1" customWidth="1"/>
-    <col min="2" max="2" width="88" style="1" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="92" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -969,7 +898,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -977,7 +906,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>47</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -985,11 +914,19 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>49</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1000,106 +937,45 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="70" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2">
         <v>5</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="76" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>68</v>
+      <c r="C3">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>